<commit_message>
Fix #VALUE! errors on Lender_Metrics summary rows
Min LLCR / Min debt yield / Max break-even occupancy / Bankability score
were written as array formulas (=MIN(IF(range<>"-",range))) which require
Ctrl+Shift+Enter to evaluate in non-dynamic-array Excel. openpyxl cannot
mark CSE formulas, so Excel returned #VALUE! on open.

MIN and MAX ignore text values natively, so the wrapping IF was
unnecessary. Replaced with direct =MIN(E10:N10), =MIN(E13:N13),
=MAX(E14:N14).

Also wrapped the Bankability score formula in IFERROR("REVIEW") so any
partial result no longer cascades into a hard error.

Applied the same simplification to QtrDebt!C19 (Min quarterly DSCR).
</commit_message>
<xml_diff>
--- a/BinAmer_Investment_Model_v5_Institutional_Hardened.xlsx
+++ b/BinAmer_Investment_Model_v5_Institutional_Hardened.xlsx
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F42"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -846,6 +846,7 @@
     <col width="18" customWidth="1" min="4" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -853,6 +854,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -913,6 +915,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="15" customHeight="1">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -980,6 +983,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1143,6 +1147,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="15" customHeight="1">
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -1288,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1301,6 +1306,7 @@
     <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -1315,6 +1321,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="58" t="inlineStr">
         <is>
@@ -1436,6 +1443,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="B17" s="53" t="inlineStr">
         <is>
@@ -1752,6 +1760,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="B25" s="53" t="inlineStr">
         <is>
@@ -1852,6 +1861,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="69" t="inlineStr">
         <is>
@@ -1914,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F33"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1925,6 +1935,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -1939,6 +1950,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="53" t="inlineStr">
         <is>
@@ -2067,6 +2079,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="53" t="inlineStr">
         <is>
@@ -2332,6 +2345,7 @@
         <v/>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="B32" s="69" t="inlineStr">
         <is>
@@ -2373,7 +2387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2382,6 +2396,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -2954,7 +2969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N26"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2963,6 +2978,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -3568,6 +3584,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -4051,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N25"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4060,6 +4077,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -4420,6 +4438,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -4580,6 +4599,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="B17" s="31" t="inlineStr">
         <is>
@@ -4607,6 +4627,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -4767,6 +4788,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
         <is>
@@ -4796,7 +4818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F36"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4806,6 +4828,7 @@
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -4813,6 +4836,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -4908,6 +4932,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -4970,6 +4995,7 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -5010,6 +5036,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="15" customHeight="1">
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -5072,6 +5099,7 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
     <row r="33" ht="15" customHeight="1">
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -5132,7 +5160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5144,6 +5172,7 @@
     <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -5158,6 +5187,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="40" t="inlineStr">
         <is>
@@ -5280,6 +5310,7 @@
         <v>-25</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -5301,6 +5332,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1">
       <c r="B16" s="31" t="inlineStr">
         <is>
@@ -5352,7 +5384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G22"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5364,6 +5396,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -5378,6 +5411,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="65" t="inlineStr">
         <is>
@@ -5626,6 +5660,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="58" t="inlineStr">
         <is>
@@ -5864,7 +5899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5873,6 +5908,7 @@
     <col width="15" customWidth="1" min="4" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -5887,6 +5923,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -5905,6 +5942,7 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="31" t="inlineStr">
         <is>
@@ -6054,6 +6092,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -6179,6 +6218,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -6291,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6307,6 +6347,7 @@
     <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -6321,6 +6362,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="53" t="inlineStr">
         <is>
@@ -6328,6 +6370,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="C7" s="86" t="n">
         <v>0.055</v>
@@ -6582,6 +6625,9 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="53" t="inlineStr">
         <is>
@@ -6589,6 +6635,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="C20" s="86" t="n">
         <v>0.055</v>
@@ -6843,6 +6890,8 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="53" t="inlineStr">
         <is>
@@ -6850,6 +6899,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="C32" s="86" t="n">
         <v>0.065</v>
@@ -7104,6 +7154,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="B41" s="52" t="inlineStr">
         <is>
@@ -7146,13 +7197,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B54"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="51" t="inlineStr">
         <is>
@@ -7167,6 +7219,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="53" t="inlineStr">
         <is>
@@ -7188,6 +7241,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="53" t="inlineStr">
         <is>
@@ -7265,6 +7319,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="B22" s="53" t="inlineStr">
         <is>
@@ -7342,6 +7398,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="B34" s="53" t="inlineStr">
         <is>
@@ -7412,6 +7469,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="B45" s="53" t="inlineStr">
         <is>
@@ -7447,6 +7505,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="B51" s="53" t="inlineStr">
         <is>
@@ -7486,7 +7545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N24"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7506,6 +7565,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -7513,6 +7573,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="D5" s="65" t="inlineStr">
         <is>
@@ -7723,6 +7785,7 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="69" t="inlineStr">
         <is>
@@ -7825,6 +7888,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="B13" s="58" t="inlineStr">
         <is>
@@ -8029,6 +8093,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="53" t="inlineStr">
         <is>
@@ -8065,7 +8130,7 @@
         </is>
       </c>
       <c r="D21" s="72">
-        <f>MIN(IF(E10:N10&lt;&gt;"-",E10:N10))</f>
+        <f>MIN(E10:N10)</f>
         <v/>
       </c>
     </row>
@@ -8076,7 +8141,7 @@
         </is>
       </c>
       <c r="D22" s="99">
-        <f>MIN(IF(E13:N13&lt;&gt;"-",E13:N13))</f>
+        <f>MIN(E13:N13)</f>
         <v/>
       </c>
     </row>
@@ -8087,7 +8152,7 @@
         </is>
       </c>
       <c r="D23" s="99">
-        <f>MAX(IF(E14:N14&lt;&gt;"-",E14:N14))</f>
+        <f>MAX(E14:N14)</f>
         <v/>
       </c>
     </row>
@@ -8098,7 +8163,7 @@
         </is>
       </c>
       <c r="D24" s="58">
-        <f>IF(AND(D20&gt;=Assumptions!$D$73,D21&gt;=1.4,D22&gt;=Assumptions!$D$75),"BANKABLE",IF(AND(D20&gt;=1.15,D21&gt;=1.20),"CONDITIONAL","NOT BANKABLE"))</f>
+        <f>IFERROR(IF(AND(D20&gt;=Assumptions!$D$73,D21&gt;=1.4,D22&gt;=Assumptions!$D$75),"BANKABLE",IF(AND(D20&gt;=1.15,D21&gt;=1.20),"CONDITIONAL","NOT BANKABLE")),"REVIEW")</f>
         <v/>
       </c>
     </row>
@@ -8124,7 +8189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I70"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8135,6 +8200,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -8149,6 +8215,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="65" t="inlineStr">
         <is>
@@ -8564,6 +8631,8 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="B25" s="53" t="inlineStr">
         <is>
@@ -8597,6 +8666,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="53" t="inlineStr">
         <is>
@@ -8674,6 +8744,16 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
     <row r="50">
       <c r="B50" s="100" t="inlineStr">
         <is>
@@ -8824,6 +8904,8 @@
         <v/>
       </c>
     </row>
+    <row r="64"/>
+    <row r="65"/>
     <row r="66">
       <c r="B66" s="100" t="inlineStr">
         <is>
@@ -9010,7 +9092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9020,6 +9102,7 @@
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -9034,6 +9117,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="40" t="inlineStr">
         <is>
@@ -9472,7 +9556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H54"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9485,6 +9569,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -9492,6 +9577,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -9587,6 +9673,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -9704,6 +9791,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="15" customHeight="1">
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -9777,6 +9865,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="15" customHeight="1">
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -9817,6 +9906,7 @@
         <v/>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="15" customHeight="1">
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -9842,6 +9932,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1">
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -9975,7 +10066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G117"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9986,6 +10077,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="57" t="inlineStr">
         <is>
@@ -10000,6 +10092,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="9" t="inlineStr">
         <is>
@@ -10068,6 +10161,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="15" customHeight="1">
       <c r="B10" s="9" t="inlineStr">
         <is>
@@ -10197,6 +10291,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
         <is>
@@ -10284,6 +10379,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="15" customHeight="1">
       <c r="B24" s="9" t="inlineStr">
         <is>
@@ -10351,6 +10447,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29" ht="15" customHeight="1">
       <c r="B29" s="9" t="inlineStr">
         <is>
@@ -10438,6 +10535,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35" ht="15" customHeight="1">
       <c r="B35" s="9" t="inlineStr">
         <is>
@@ -10505,6 +10603,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="15" customHeight="1">
       <c r="B40" s="9" t="inlineStr">
         <is>
@@ -10674,6 +10773,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1">
       <c r="B50" s="9" t="inlineStr">
         <is>
@@ -10761,6 +10861,7 @@
         </is>
       </c>
     </row>
+    <row r="55"/>
     <row r="56" ht="15" customHeight="1">
       <c r="B56" s="9" t="inlineStr">
         <is>
@@ -10848,6 +10949,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="15" customHeight="1">
       <c r="B62" s="9" t="inlineStr">
         <is>
@@ -10978,6 +11080,7 @@
         </is>
       </c>
     </row>
+    <row r="69"/>
     <row r="70" ht="15" customHeight="1">
       <c r="B70" s="9" t="inlineStr">
         <is>
@@ -11294,6 +11397,7 @@
         </is>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="B88" s="53" t="inlineStr">
         <is>
@@ -11401,6 +11505,7 @@
         </is>
       </c>
     </row>
+    <row r="94"/>
     <row r="95">
       <c r="B95" s="53" t="inlineStr">
         <is>
@@ -11623,6 +11728,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="106"/>
     <row r="107">
       <c r="B107" s="69" t="inlineStr">
         <is>
@@ -11643,6 +11749,7 @@
         </is>
       </c>
     </row>
+    <row r="108"/>
     <row r="109">
       <c r="B109" s="53" t="inlineStr">
         <is>
@@ -11836,7 +11943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11845,6 +11952,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -12206,7 +12314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -12215,6 +12323,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -12529,7 +12638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N23"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -12538,6 +12647,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -12898,6 +13008,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -13211,6 +13322,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -13389,7 +13501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -13398,6 +13510,7 @@
     <col width="13" customWidth="1" min="4" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="27.75" customHeight="1">
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -13880,6 +13993,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -14158,7 +14272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AQ20"/>
+  <dimension ref="A1:AQ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -14207,6 +14321,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="73" t="inlineStr">
         <is>
@@ -14221,6 +14336,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="65" t="inlineStr">
         <is>
@@ -14775,6 +14891,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="58" t="inlineStr">
         <is>
@@ -15761,6 +15878,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="B16" s="69" t="inlineStr">
         <is>
@@ -16103,6 +16221,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" s="69" t="inlineStr">
         <is>
@@ -16110,7 +16229,7 @@
         </is>
       </c>
       <c r="C19" s="76">
-        <f>IFERROR(MIN(IF(C16:AQ16&lt;&gt;"-",C16:AQ16)),0)</f>
+        <f>MIN(C16:AQ16)</f>
         <v/>
       </c>
     </row>

</xml_diff>